<commit_message>
Revisions in Client Records
</commit_message>
<xml_diff>
--- a/capstone-project/public/Export_Template_Referred.xlsx
+++ b/capstone-project/public/Export_Template_Referred.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lheriza Miranda\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A7732EFE-C55A-49D7-B0B4-72BBC01E7F2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCEADACB-6DB4-45E8-A317-E6AB0CD07D51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6BB6BB68-EF4E-424F-9D07-CD80EE37AB5A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{6BB6BB68-EF4E-424F-9D07-CD80EE37AB5A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -65,14 +65,14 @@
     <t>Date</t>
   </si>
   <si>
-    <t>Referred and Served List</t>
+    <t>Referred and Served List Users</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -80,13 +80,35 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0627A2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -116,17 +138,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -134,6 +160,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF0627A2"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -143,6 +174,100 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>137160</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>760300</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>99060</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{37432DB9-E20B-4716-AC14-70F108F7D799}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4175760" y="76200"/>
+          <a:ext cx="623140" cy="571500"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>571500</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>1280448</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>121920</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{56E7CC7E-C327-4695-8CF3-5EC524E63D8A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
+        <a:srcRect t="13212" b="17202"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8001000" y="30480"/>
+          <a:ext cx="708948" cy="640080"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -468,48 +593,48 @@
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="4.44140625" customWidth="1"/>
     <col min="3" max="3" width="21.21875" customWidth="1"/>
-    <col min="4" max="4" width="25.21875" customWidth="1"/>
+    <col min="4" max="4" width="29.33203125" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="23.21875" customWidth="1"/>
-    <col min="7" max="7" width="23.44140625" customWidth="1"/>
+    <col min="6" max="6" width="33.33203125" customWidth="1"/>
+    <col min="7" max="7" width="31.88671875" customWidth="1"/>
     <col min="8" max="8" width="19.5546875" customWidth="1"/>
-    <col min="9" max="9" width="18.44140625" customWidth="1"/>
+    <col min="9" max="9" width="22.5546875" customWidth="1"/>
     <col min="10" max="10" width="15.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:10" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
     </row>
-    <row r="4" spans="2:10" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B4" s="1"/>
-      <c r="C4" s="2" t="s">
+    <row r="4" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B4" s="4"/>
+      <c r="C4" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="J4" s="5" t="s">
         <v>7</v>
       </c>
     </row>
@@ -532,5 +657,6 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>